<commit_message>
JsonManager 및 TC 갱신 , 코드 수정
몬스터 Data 추가,
몬스터 패시브 옵션 Data 추가,
JsonManager 권한 분할(하나의 코드에 너무 많은 권한이 들어있음)
RemoteTester의 기능 추가
등등
</commit_message>
<xml_diff>
--- a/JsonFile/memory/TC_List.xlsx
+++ b/JsonFile/memory/TC_List.xlsx
@@ -109,7 +109,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -146,11 +146,25 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -174,6 +188,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -5740,22 +5757,22 @@
   <dimension ref="A1:P51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="38" customWidth="1" min="5" max="5"/>
-    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
     <col width="34" customWidth="1" min="7" max="7"/>
-    <col width="46" customWidth="1" min="8" max="8"/>
-    <col width="36" customWidth="1" min="9" max="9"/>
-    <col width="38" customWidth="1" min="10" max="10"/>
-    <col width="38" customWidth="1" min="11" max="11"/>
+    <col width="48" customWidth="1" min="8" max="8"/>
+    <col width="42" customWidth="1" min="9" max="9"/>
+    <col width="42" customWidth="1" min="10" max="10"/>
+    <col width="36" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="36" customWidth="1" min="13" max="13"/>
-    <col width="34" customWidth="1" min="14" max="14"/>
-    <col width="14" customWidth="1" min="15" max="15"/>
-    <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="34" customWidth="1" min="13" max="13"/>
+    <col width="32" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -5840,113 +5857,515 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="8" t="n"/>
-      <c r="B2" s="8" t="n"/>
-      <c r="C2" s="8" t="n"/>
-      <c r="D2" s="8" t="n"/>
-      <c r="E2" s="8" t="n"/>
-      <c r="F2" s="8" t="n"/>
-      <c r="G2" s="8" t="n"/>
-      <c r="H2" s="8" t="n"/>
-      <c r="I2" s="8" t="n"/>
-      <c r="J2" s="8" t="n"/>
-      <c r="K2" s="8" t="n"/>
-      <c r="L2" s="8" t="n"/>
-      <c r="M2" s="8" t="n"/>
-      <c r="N2" s="8" t="n"/>
-      <c r="O2" s="8" t="n"/>
-      <c r="P2" s="8" t="n"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="8" t="n"/>
-      <c r="B3" s="8" t="n"/>
-      <c r="C3" s="8" t="n"/>
-      <c r="D3" s="8" t="n"/>
-      <c r="E3" s="8" t="n"/>
-      <c r="F3" s="8" t="n"/>
-      <c r="G3" s="8" t="n"/>
-      <c r="H3" s="8" t="n"/>
-      <c r="I3" s="8" t="n"/>
-      <c r="J3" s="8" t="n"/>
-      <c r="K3" s="8" t="n"/>
-      <c r="L3" s="8" t="n"/>
-      <c r="M3" s="8" t="n"/>
-      <c r="N3" s="8" t="n"/>
-      <c r="O3" s="8" t="n"/>
-      <c r="P3" s="8" t="n"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="8" t="n"/>
-      <c r="B4" s="8" t="n"/>
-      <c r="C4" s="8" t="n"/>
-      <c r="D4" s="8" t="n"/>
-      <c r="E4" s="8" t="n"/>
-      <c r="F4" s="8" t="n"/>
-      <c r="G4" s="8" t="n"/>
-      <c r="H4" s="8" t="n"/>
-      <c r="I4" s="8" t="n"/>
-      <c r="J4" s="8" t="n"/>
-      <c r="K4" s="8" t="n"/>
-      <c r="L4" s="8" t="n"/>
-      <c r="M4" s="8" t="n"/>
-      <c r="N4" s="8" t="n"/>
-      <c r="O4" s="8" t="n"/>
-      <c r="P4" s="8" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="8" t="n"/>
-      <c r="B5" s="8" t="n"/>
-      <c r="C5" s="8" t="n"/>
-      <c r="D5" s="8" t="n"/>
-      <c r="E5" s="8" t="n"/>
-      <c r="F5" s="8" t="n"/>
-      <c r="G5" s="8" t="n"/>
-      <c r="H5" s="8" t="n"/>
-      <c r="I5" s="8" t="n"/>
-      <c r="J5" s="8" t="n"/>
-      <c r="K5" s="8" t="n"/>
-      <c r="L5" s="8" t="n"/>
-      <c r="M5" s="8" t="n"/>
-      <c r="N5" s="8" t="n"/>
-      <c r="O5" s="8" t="n"/>
-      <c r="P5" s="8" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="8" t="n"/>
-      <c r="B6" s="8" t="n"/>
-      <c r="C6" s="8" t="n"/>
-      <c r="D6" s="8" t="n"/>
-      <c r="E6" s="8" t="n"/>
-      <c r="F6" s="8" t="n"/>
-      <c r="G6" s="8" t="n"/>
-      <c r="H6" s="8" t="n"/>
-      <c r="I6" s="8" t="n"/>
-      <c r="J6" s="8" t="n"/>
-      <c r="K6" s="8" t="n"/>
-      <c r="L6" s="8" t="n"/>
-      <c r="M6" s="8" t="n"/>
-      <c r="N6" s="8" t="n"/>
-      <c r="O6" s="8" t="n"/>
-      <c r="P6" s="8" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="8" t="n"/>
-      <c r="B7" s="8" t="n"/>
-      <c r="C7" s="8" t="n"/>
-      <c r="D7" s="8" t="n"/>
-      <c r="E7" s="8" t="n"/>
-      <c r="F7" s="8" t="n"/>
-      <c r="G7" s="8" t="n"/>
-      <c r="H7" s="8" t="n"/>
-      <c r="I7" s="8" t="n"/>
-      <c r="J7" s="8" t="n"/>
-      <c r="K7" s="8" t="n"/>
-      <c r="L7" s="8" t="n"/>
-      <c r="M7" s="8" t="n"/>
-      <c r="N7" s="8" t="n"/>
-      <c r="O7" s="8" t="n"/>
-      <c r="P7" s="8" t="n"/>
+    <row r="2" ht="78" customHeight="1">
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>MTC-MON-001</t>
+        </is>
+      </c>
+      <c r="B2" s="9" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C2" s="9" t="inlineStr">
+        <is>
+          <t>몬스터 옵션 브릿지 기본 수집 검증</t>
+        </is>
+      </c>
+      <c r="D2" s="9" t="inlineStr">
+        <is>
+          <t>전투/데이터</t>
+        </is>
+      </c>
+      <c r="E2" s="9" t="inlineStr">
+        <is>
+          <t>MonPas_EffectN 슬롯이 고정 2개에 묶이지 않고 몬스터 옵션으로 등록되는지 확인한다.</t>
+        </is>
+      </c>
+      <c r="F2" s="9" t="inlineStr">
+        <is>
+          <t>Unity Editor에서 JsonFile 프로젝트가 컴파일 완료 상태이며 RemoteTester 또는 전투 진입 경로를 사용할 수 있다.</t>
+        </is>
+      </c>
+      <c r="G2" s="9" t="inlineStr">
+        <is>
+          <t>Mon_Master: monster_002, monster_007, monster_010 / Effect*_Stat=0</t>
+        </is>
+      </c>
+      <c r="H2" s="9" t="inlineStr">
+        <is>
+          <t>1. 에디터에서 테스트 전투 메뉴를 연다.
+2. monster_002, monster_007, monster_010을 순서대로 선택한다.
+3. 전투 시작 직후 Console과 전투 UI 상태를 확인한다.
+4. 미등록 옵션 또는 MonEffect_000 경고가 발생하는지 확인한다.</t>
+        </is>
+      </c>
+      <c r="I2" s="9" t="inlineStr">
+        <is>
+          <t>Console에 미등록 Option 경고가 없는지, 각 몬스터의 옵션 개수가 의도대로 등록되는지, 전투 시작이 중단되지 않는지 확인한다.</t>
+        </is>
+      </c>
+      <c r="J2" s="9" t="inlineStr">
+        <is>
+          <t>MonPas_EffectN 기반 옵션이 정상 등록되고 NoOp 값은 조용히 무시된다.</t>
+        </is>
+      </c>
+      <c r="K2" s="9" t="inlineStr">
+        <is>
+          <t>자동 EditMode 사전 검증: 41/41 통과. 수동 플레이테스트 미실행.</t>
+        </is>
+      </c>
+      <c r="L2" s="9" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+      <c r="M2" s="9" t="inlineStr">
+        <is>
+          <t>슬롯 확장성 확인용. 보스용 MonPas_Effect3+ 추가 전 회귀 테스트로 유지.</t>
+        </is>
+      </c>
+      <c r="N2" s="9" t="inlineStr">
+        <is>
+          <t>수동 확인 시 Console Warning/Log 캡처 권장.</t>
+        </is>
+      </c>
+      <c r="O2" s="9" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="P2" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="78" customHeight="1">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>MTC-MON-002</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C3" s="9" t="inlineStr">
+        <is>
+          <t>몬스터 OnHit 출혈/독 적용 확인</t>
+        </is>
+      </c>
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>전투/상태이상</t>
+        </is>
+      </c>
+      <c r="E3" s="9" t="inlineStr">
+        <is>
+          <t>몬스터가 기존 OptionManager의 OnHit 상태이상 효과를 재사용하는지 확인한다.</t>
+        </is>
+      </c>
+      <c r="F3" s="9" t="inlineStr">
+        <is>
+          <t>플레이어가 monster_002 또는 monster_009와 전투 가능해야 한다.</t>
+        </is>
+      </c>
+      <c r="G3" s="9" t="inlineStr">
+        <is>
+          <t>monster_002: Option_009, Option_010 / monster_009: Option_010 / Effect*_Stat=0</t>
+        </is>
+      </c>
+      <c r="H3" s="9" t="inlineStr">
+        <is>
+          <t>1. monster_002와 전투를 시작한다.
+2. 몬스터가 플레이어를 3회 이상 공격하도록 진행한다.
+3. 플레이어 버프/디버프 UI와 HP 변화를 관찰한다.
+4. monster_009로 동일 절차를 반복한다.</t>
+        </is>
+      </c>
+      <c r="I3" s="9" t="inlineStr">
+        <is>
+          <t>출혈 또는 독 스택이 플레이어에게 적용되는지, 스택 증가/틱 피해가 기존 장비 옵션과 동일한 규칙을 따르는지 확인한다.</t>
+        </is>
+      </c>
+      <c r="J3" s="9" t="inlineStr">
+        <is>
+          <t>몬스터 적중 시 출혈/독 디버프가 적용되고 전투 진행을 막는 예외가 없다.</t>
+        </is>
+      </c>
+      <c r="K3" s="9" t="inlineStr">
+        <is>
+          <t>자동 EditMode 사전 검증: 41/41 통과. 수동 플레이테스트 미실행.</t>
+        </is>
+      </c>
+      <c r="L3" s="9" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+      <c r="M3" s="9" t="inlineStr">
+        <is>
+          <t>피해량 밸런스는 확정하지 않는다. 적용 여부와 스택 동작만 확인.</t>
+        </is>
+      </c>
+      <c r="N3" s="9" t="inlineStr">
+        <is>
+          <t>값은 추후 밸런스 자동화 후 조정.</t>
+        </is>
+      </c>
+      <c r="O3" s="9" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="P3" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="78" customHeight="1">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>MTC-MON-003</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>몬스터 강제 빗나감 효과 확인</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>전투/상태이상</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>몬스터 OnHit Option_008이 플레이어의 다음 공격 실패 상태를 정상 부여하는지 확인한다.</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>플레이어가 monster_005 또는 monster_007과 전투 가능해야 한다.</t>
+        </is>
+      </c>
+      <c r="G4" s="9" t="inlineStr">
+        <is>
+          <t>monster_005: Option_008 / monster_007: Option_008 + Option_009</t>
+        </is>
+      </c>
+      <c r="H4" s="9" t="inlineStr">
+        <is>
+          <t>1. monster_005와 전투를 시작한다.
+2. 몬스터 공격이 적중한 뒤 플레이어의 다음 공격 결과를 확인한다.
+3. CombatFeedback 또는 로그에서 공격 실패 처리가 1회만 소비되는지 확인한다.
+4. monster_007에서도 동일하게 확인한다.</t>
+        </is>
+      </c>
+      <c r="I4" s="9" t="inlineStr">
+        <is>
+          <t>강제 빗나감이 1회 적용 후 소비되는지, 출혈과 함께 있어도 서로 막지 않는지 확인한다.</t>
+        </is>
+      </c>
+      <c r="J4" s="9" t="inlineStr">
+        <is>
+          <t>몬스터 적중 후 플레이어 다음 공격이 1회 실패하고 이후 정상 공격으로 복귀한다.</t>
+        </is>
+      </c>
+      <c r="K4" s="9" t="inlineStr">
+        <is>
+          <t>자동 EditMode 사전 검증: 41/41 통과. 수동 플레이테스트 미실행.</t>
+        </is>
+      </c>
+      <c r="L4" s="9" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+      <c r="M4" s="9" t="inlineStr">
+        <is>
+          <t>확률이 아닌 상태 부여/소비 흐름 중심 확인.</t>
+        </is>
+      </c>
+      <c r="N4" s="9" t="inlineStr">
+        <is>
+          <t>공격 순서에 따라 재현 타이밍이 달라질 수 있음.</t>
+        </is>
+      </c>
+      <c r="O4" s="9" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="P4" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="78" customHeight="1">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>MTC-MON-004</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>몬스터 BattleStart 패시브 임시 적용/정리 확인</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>전투/패시브</t>
+        </is>
+      </c>
+      <c r="E5" s="9" t="inlineStr">
+        <is>
+          <t>몬스터 패시브가 전투 시작 시 적용되고 전투 종료 후 남지 않는지 확인한다.</t>
+        </is>
+      </c>
+      <c r="F5" s="9" t="inlineStr">
+        <is>
+          <t>monster_008 또는 monster_010과 전투를 시작하고 종료할 수 있어야 한다.</t>
+        </is>
+      </c>
+      <c r="G5" s="9" t="inlineStr">
+        <is>
+          <t>monster_008: Option_014 / monster_010: Option_013 + Option_018</t>
+        </is>
+      </c>
+      <c r="H5" s="9" t="inlineStr">
+        <is>
+          <t>1. monster_008 전투 시작 직후 몬스터 상태/로그를 확인한다.
+2. 전투를 승리 또는 패배로 종료한다.
+3. 다음 전투에 진입해 이전 전투의 몬스터 패시브가 남아 있지 않은지 확인한다.
+4. monster_010으로 광폭화/빙결 조합도 반복 확인한다.</t>
+        </is>
+      </c>
+      <c r="I5" s="9" t="inlineStr">
+        <is>
+          <t>전투 시작 패시브가 한 전투 동안만 유지되는지, RemoveTemporaryBuffs 이후 스탯이 복구되는지 확인한다.</t>
+        </is>
+      </c>
+      <c r="J5" s="9" t="inlineStr">
+        <is>
+          <t>몬스터 패시브는 전투 종료 시 정리되고 다음 전투에 누적되지 않는다.</t>
+        </is>
+      </c>
+      <c r="K5" s="9" t="inlineStr">
+        <is>
+          <t>자동 EditMode 사전 검증: 41/41 통과. 수동 플레이테스트 미실행.</t>
+        </is>
+      </c>
+      <c r="L5" s="9" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+      <c r="M5" s="9" t="inlineStr">
+        <is>
+          <t>장비 패시브와 달리 몬스터 패시브는 저장/장착 상태로 남으면 안 됨.</t>
+        </is>
+      </c>
+      <c r="N5" s="9" t="inlineStr">
+        <is>
+          <t>전투 종료 UI 팝업 이후 재진입까지 확인 필요.</t>
+        </is>
+      </c>
+      <c r="O5" s="9" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="P5" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="78" customHeight="1">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>MTC-MON-005</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>몬스터 빙결/광폭화 복합 효과 확인</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>전투/복합 효과</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>상위 몬스터가 여러 효과를 동시에 가져도 전투 흐름과 UI가 깨지지 않는지 확인한다.</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>monster_010 전투 가능 상태. 플레이어 HP/정신력이 전투 진행 가능한 값이어야 한다.</t>
+        </is>
+      </c>
+      <c r="G6" s="9" t="inlineStr">
+        <is>
+          <t>monster_010: Option_013, Option_018 / Effect*_Stat=0</t>
+        </is>
+      </c>
+      <c r="H6" s="9" t="inlineStr">
+        <is>
+          <t>1. monster_010과 전투를 시작한다.
+2. 전투 시작 직후 광폭화 관련 스탯 변화가 적용되는지 확인한다.
+3. 몬스터 적중 후 빙결 디버프가 플레이어에게 적용되는지 확인한다.
+4. 전투 종료 후 재전투에서 효과가 중복 누적되지 않는지 확인한다.</t>
+        </is>
+      </c>
+      <c r="I6" s="9" t="inlineStr">
+        <is>
+          <t>광폭화와 빙결이 같은 몬스터에 있어도 각각 올바른 트리거에서 실행되는지 확인한다.</t>
+        </is>
+      </c>
+      <c r="J6" s="9" t="inlineStr">
+        <is>
+          <t>전투 시작 효과와 적중 효과가 분리되어 실행되고 중복 누적/잔류가 없다.</t>
+        </is>
+      </c>
+      <c r="K6" s="9" t="inlineStr">
+        <is>
+          <t>자동 EditMode 사전 검증: 41/41 통과. 수동 플레이테스트 미실행.</t>
+        </is>
+      </c>
+      <c r="L6" s="9" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+      <c r="M6" s="9" t="inlineStr">
+        <is>
+          <t>보스 몬스터 다중 패시브 확장 전 대표 시나리오.</t>
+        </is>
+      </c>
+      <c r="N6" s="9" t="inlineStr">
+        <is>
+          <t>체감 난이도는 추후 별도 밸런스 TC로 분리.</t>
+        </is>
+      </c>
+      <c r="O6" s="9" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="P6" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="78" customHeight="1">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>MTC-MON-006</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>몬스터 옵션 데이터 무결성 회귀 확인</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>데이터/회귀</t>
+        </is>
+      </c>
+      <c r="E7" s="9" t="inlineStr">
+        <is>
+          <t>Mon_Master에 입력된 Option_* 또는 MonEffect_* ID가 런타임에서 모두 해석 가능한지 확인한다.</t>
+        </is>
+      </c>
+      <c r="F7" s="9" t="inlineStr">
+        <is>
+          <t>Excel Auto Generator를 다시 실행했거나 몬스터 데이터가 변경된 이후 수행한다.</t>
+        </is>
+      </c>
+      <c r="G7" s="9" t="inlineStr">
+        <is>
+          <t>Monster_Data.xlsx, Mon_Master.json, Option_Master.json, Mon_Effect_Master.json</t>
+        </is>
+      </c>
+      <c r="H7" s="9" t="inlineStr">
+        <is>
+          <t>1. Excel Auto Generator를 실행한 뒤 Unity 컴파일 완료를 기다린다.
+2. EditMode 테스트를 실행한다.
+3. Mon_Master 관련 데이터 검증 실패 또는 미등록 옵션 경고가 없는지 확인한다.
+4. 몬스터 이름 한글 깨짐 여부도 함께 확인한다.</t>
+        </is>
+      </c>
+      <c r="I7" s="9" t="inlineStr">
+        <is>
+          <t>Option_*는 Option_Master에 존재하고 MonEffect_*는 MonsterOptionManager에 등록되어 있는지 확인한다.</t>
+        </is>
+      </c>
+      <c r="J7" s="9" t="inlineStr">
+        <is>
+          <t>데이터 재생성 후에도 몬스터 옵션 ID와 한글 이름이 유지된다.</t>
+        </is>
+      </c>
+      <c r="K7" s="9" t="inlineStr">
+        <is>
+          <t>자동 EditMode 사전 검증: 41/41 통과. 수동 플레이테스트 미실행.</t>
+        </is>
+      </c>
+      <c r="L7" s="9" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+      <c r="M7" s="9" t="inlineStr">
+        <is>
+          <t>엑셀 변환기 한글/타입 추론 이슈 회귀 방지용.</t>
+        </is>
+      </c>
+      <c r="N7" s="9" t="inlineStr">
+        <is>
+          <t>Effect*_Stat는 0이어도 미밸런싱 값으로 허용.</t>
+        </is>
+      </c>
+      <c r="O7" s="9" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="P7" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="n"/>

</xml_diff>